<commit_message>
fix: consolidar ativos por ticker normalizado e corrigir parsing de datas
- ativos.py: corrige regex de ticker para capturar B3SA3 corretamente e
  preservar ativos sem código (Tesouro Direto)
- eventos.py: aplicar_eventos_ordenados agora agrupa por renomear_ativo,
  eliminando duplicação causada por variações de nome do mesmo ativo
  (ex: PETR4 com duas grafias) e unificando histórico NUBR33/NUBR35/ROXO34
- movimentacao.py: fallback de parsing de datas com format='mixed' para
  aceitar datas fora do padrão dd/mm/yyyy sem gerar NaT
- fixture movimentacao_7_ativos.xlsx: inseridas linhas reais da migração
  Nubank (NUBR33 débito, NUBR35 crédito, ROXO34 atualização) em 15/08/2023
  na posição cronológica correta e removidas duplicatas do final

Todos os 83 testes passando + 1 xfail esperado (ROXO34 custo sem origem)
</commit_message>
<xml_diff>
--- a/tests/fixtures/movimentacao_7_ativos.xlsx
+++ b/tests/fixtures/movimentacao_7_ativos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H236"/>
+  <dimension ref="A1:H238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6285,7 +6285,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Credito</t>
+          <t>Debito</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -6295,12 +6295,12 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Atualização</t>
+          <t>Transferência</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROXO34 - NU HOLDINGS </t>
+          <t>NUBR33 - NU HOLDINGS LTD.</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -6330,17 +6330,17 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>13/07/2023</t>
+          <t>15/08/2023</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Transferência - Liquidação</t>
+          <t>Transferência</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>VALE3 - VALE S.A.</t>
+          <t>NUBR35 - NU HOLDINGS LTD.</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -6349,13 +6349,17 @@
         </is>
       </c>
       <c r="F163" t="n">
-        <v>4</v>
-      </c>
-      <c r="G163" t="n">
-        <v>66.23</v>
-      </c>
-      <c r="H163" t="n">
-        <v>264.92</v>
+        <v>20</v>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="164">
@@ -6366,17 +6370,17 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>07/07/2023</t>
+          <t>15/08/2023</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Juros Sobre Capital Próprio</t>
+          <t>Atualização</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
+          <t>ROXO34 - NU HOLDINGS</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -6385,13 +6389,17 @@
         </is>
       </c>
       <c r="F164" t="n">
-        <v>52</v>
-      </c>
-      <c r="G164" t="n">
-        <v>0.062</v>
-      </c>
-      <c r="H164" t="n">
-        <v>2.72</v>
+        <v>20</v>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="165">
@@ -6402,17 +6410,17 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>07/07/2023</t>
+          <t>13/07/2023</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Transferência - Liquidação</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
+          <t>VALE3 - VALE S.A.</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -6421,13 +6429,13 @@
         </is>
       </c>
       <c r="F165" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="G165" t="n">
-        <v>0.054</v>
+        <v>66.23</v>
       </c>
       <c r="H165" t="n">
-        <v>2.79</v>
+        <v>264.92</v>
       </c>
     </row>
     <row r="166">
@@ -6438,17 +6446,17 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>23/06/2023</t>
+          <t>07/07/2023</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Juros Sobre Capital Próprio</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>CPFE3 - CPFL ENERGIA S/A</t>
+          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -6457,13 +6465,13 @@
         </is>
       </c>
       <c r="F166" t="n">
-        <v>3</v>
+        <v>52</v>
       </c>
       <c r="G166" t="n">
-        <v>0.54</v>
+        <v>0.062</v>
       </c>
       <c r="H166" t="n">
-        <v>1.62</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="167">
@@ -6474,17 +6482,17 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>16/06/2023</t>
+          <t>07/07/2023</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Rendimento</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -6493,13 +6501,13 @@
         </is>
       </c>
       <c r="F167" t="n">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="G167" t="n">
-        <v>0.052</v>
+        <v>0.054</v>
       </c>
       <c r="H167" t="n">
-        <v>0.68</v>
+        <v>2.79</v>
       </c>
     </row>
     <row r="168">
@@ -6510,7 +6518,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>16/06/2023</t>
+          <t>23/06/2023</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -6520,7 +6528,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t>CPFE3 - CPFL ENERGIA S/A</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -6529,13 +6537,13 @@
         </is>
       </c>
       <c r="F168" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="G168" t="n">
-        <v>0.875</v>
+        <v>0.54</v>
       </c>
       <c r="H168" t="n">
-        <v>14.87</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="169">
@@ -6546,17 +6554,17 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>14/06/2023</t>
+          <t>16/06/2023</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Rendimento</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -6565,13 +6573,13 @@
         </is>
       </c>
       <c r="F169" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G169" t="n">
-        <v>0.094</v>
+        <v>0.052</v>
       </c>
       <c r="H169" t="n">
-        <v>1.03</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="170">
@@ -6582,12 +6590,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>02/06/2023</t>
+          <t>16/06/2023</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Transferência - Liquidação</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -6601,13 +6609,13 @@
         </is>
       </c>
       <c r="F170" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="G170" t="n">
-        <v>26.26</v>
+        <v>0.875</v>
       </c>
       <c r="H170" t="n">
-        <v>26.26</v>
+        <v>14.87</v>
       </c>
     </row>
     <row r="171">
@@ -6618,17 +6626,17 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>19/05/2023</t>
+          <t>14/06/2023</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Rendimento</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -6637,13 +6645,13 @@
         </is>
       </c>
       <c r="F171" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G171" t="n">
-        <v>0.068</v>
+        <v>0.094</v>
       </c>
       <c r="H171" t="n">
-        <v>0.89</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="172">
@@ -6654,12 +6662,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>19/05/2023</t>
+          <t>02/06/2023</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Transferência - Liquidação</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -6673,13 +6681,13 @@
         </is>
       </c>
       <c r="F172" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="G172" t="n">
-        <v>1.373</v>
+        <v>26.26</v>
       </c>
       <c r="H172" t="n">
-        <v>23.33</v>
+        <v>26.26</v>
       </c>
     </row>
     <row r="173">
@@ -6690,17 +6698,17 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>16/05/2023</t>
+          <t>19/05/2023</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Rendimento</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>CPFE3 - CPFL ENERGIA S/A</t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
@@ -6709,13 +6717,13 @@
         </is>
       </c>
       <c r="F173" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="G173" t="n">
-        <v>0.868</v>
+        <v>0.068</v>
       </c>
       <c r="H173" t="n">
-        <v>2.6</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="174">
@@ -6726,7 +6734,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>10/04/2023</t>
+          <t>19/05/2023</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -6736,7 +6744,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
@@ -6745,13 +6753,13 @@
         </is>
       </c>
       <c r="F174" t="n">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="G174" t="n">
-        <v>0.037</v>
+        <v>1.373</v>
       </c>
       <c r="H174" t="n">
-        <v>1.9</v>
+        <v>23.33</v>
       </c>
     </row>
     <row r="175">
@@ -6762,17 +6770,17 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>10/04/2023</t>
+          <t>16/05/2023</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Juros Sobre Capital Próprio</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
+          <t>CPFE3 - CPFL ENERGIA S/A</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -6781,13 +6789,13 @@
         </is>
       </c>
       <c r="F175" t="n">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="G175" t="n">
-        <v>0.06</v>
+        <v>0.868</v>
       </c>
       <c r="H175" t="n">
-        <v>2.66</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="176">
@@ -6798,17 +6806,17 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>22/03/2023</t>
+          <t>10/04/2023</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Juros Sobre Capital Próprio</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>VALE3 - VALE S.A.</t>
+          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
@@ -6817,13 +6825,13 @@
         </is>
       </c>
       <c r="F176" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="G176" t="n">
-        <v>0.292</v>
+        <v>0.037</v>
       </c>
       <c r="H176" t="n">
-        <v>0.99</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="177">
@@ -6834,17 +6842,17 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>22/03/2023</t>
+          <t>10/04/2023</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Juros Sobre Capital Próprio</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>VALE3 - VALE S.A.</t>
+          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -6853,13 +6861,13 @@
         </is>
       </c>
       <c r="F177" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="G177" t="n">
-        <v>1.828</v>
+        <v>0.06</v>
       </c>
       <c r="H177" t="n">
-        <v>7.31</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="178">
@@ -6870,17 +6878,17 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>15/03/2023</t>
+          <t>22/03/2023</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Juros Sobre Capital Próprio</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>VALE3 - VALE S.A.</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
@@ -6889,13 +6897,13 @@
         </is>
       </c>
       <c r="F178" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="G178" t="n">
-        <v>0.099</v>
+        <v>0.292</v>
       </c>
       <c r="H178" t="n">
-        <v>1.09</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="179">
@@ -6906,17 +6914,17 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>27/02/2023</t>
+          <t>22/03/2023</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Transferência - Liquidação</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
+          <t>VALE3 - VALE S.A.</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
@@ -6925,13 +6933,13 @@
         </is>
       </c>
       <c r="F179" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G179" t="n">
-        <v>10.875</v>
+        <v>1.828</v>
       </c>
       <c r="H179" t="n">
-        <v>21.75</v>
+        <v>7.31</v>
       </c>
     </row>
     <row r="180">
@@ -6942,17 +6950,17 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>27/02/2023</t>
+          <t>15/03/2023</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Transferência - Liquidação</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>CPFE3 - CPFL ENERGIA S/A</t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -6961,13 +6969,13 @@
         </is>
       </c>
       <c r="F180" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G180" t="n">
-        <v>30.78</v>
+        <v>0.099</v>
       </c>
       <c r="H180" t="n">
-        <v>92.34</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="181">
@@ -6988,7 +6996,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -6997,13 +7005,13 @@
         </is>
       </c>
       <c r="F181" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G181" t="n">
-        <v>26.44</v>
+        <v>10.875</v>
       </c>
       <c r="H181" t="n">
-        <v>26.44</v>
+        <v>21.75</v>
       </c>
     </row>
     <row r="182">
@@ -7014,17 +7022,17 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>19/01/2023</t>
+          <t>27/02/2023</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Rendimento</t>
+          <t>Transferência - Liquidação</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t>CPFE3 - CPFL ENERGIA S/A</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
@@ -7033,13 +7041,13 @@
         </is>
       </c>
       <c r="F182" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="G182" t="n">
-        <v>0.011</v>
+        <v>30.78</v>
       </c>
       <c r="H182" t="n">
-        <v>0.14</v>
+        <v>92.34</v>
       </c>
     </row>
     <row r="183">
@@ -7050,12 +7058,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>19/01/2023</t>
+          <t>27/02/2023</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Transferência - Liquidação</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -7069,13 +7077,13 @@
         </is>
       </c>
       <c r="F183" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G183" t="n">
-        <v>1.6</v>
+        <v>26.44</v>
       </c>
       <c r="H183" t="n">
-        <v>25.6</v>
+        <v>26.44</v>
       </c>
     </row>
     <row r="184">
@@ -7091,7 +7099,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Juros Sobre Capital Próprio</t>
+          <t>Rendimento</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -7108,10 +7116,10 @@
         <v>16</v>
       </c>
       <c r="G184" t="n">
-        <v>0.074</v>
+        <v>0.011</v>
       </c>
       <c r="H184" t="n">
-        <v>1</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="185">
@@ -7122,17 +7130,17 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>13/01/2023</t>
+          <t>19/01/2023</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Juros Sobre Capital Próprio</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t xml:space="preserve">B3SA3 - B3          </t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
@@ -7141,13 +7149,13 @@
         </is>
       </c>
       <c r="F185" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="G185" t="n">
-        <v>0.064</v>
+        <v>1.6</v>
       </c>
       <c r="H185" t="n">
-        <v>2.71</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="186">
@@ -7158,17 +7166,17 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>29/12/2022</t>
+          <t>19/01/2023</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Juros Sobre Capital Próprio</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t xml:space="preserve">B3SA3 - B3          </t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -7177,13 +7185,13 @@
         </is>
       </c>
       <c r="F186" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="G186" t="n">
-        <v>0.024</v>
+        <v>0.074</v>
       </c>
       <c r="H186" t="n">
-        <v>1.21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="187">
@@ -7194,7 +7202,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>20/12/2022</t>
+          <t>13/01/2023</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -7204,7 +7212,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t xml:space="preserve">B3SA3 - B3          </t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -7213,13 +7221,13 @@
         </is>
       </c>
       <c r="F187" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="G187" t="n">
-        <v>0.519</v>
+        <v>0.064</v>
       </c>
       <c r="H187" t="n">
-        <v>7.05</v>
+        <v>2.71</v>
       </c>
     </row>
     <row r="188">
@@ -7230,7 +7238,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>20/12/2022</t>
+          <t>29/12/2022</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -7240,7 +7248,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t xml:space="preserve">B3SA3 - B3          </t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
@@ -7249,13 +7257,13 @@
         </is>
       </c>
       <c r="F188" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="G188" t="n">
-        <v>1.156</v>
+        <v>0.024</v>
       </c>
       <c r="H188" t="n">
-        <v>18.49</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="189">
@@ -7266,17 +7274,17 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>14/12/2022</t>
+          <t>20/12/2022</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Juros Sobre Capital Próprio</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -7285,13 +7293,13 @@
         </is>
       </c>
       <c r="F189" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G189" t="n">
-        <v>0.1</v>
+        <v>0.519</v>
       </c>
       <c r="H189" t="n">
-        <v>1.1</v>
+        <v>7.05</v>
       </c>
     </row>
     <row r="190">
@@ -7302,7 +7310,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>07/10/2022</t>
+          <t>20/12/2022</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -7312,7 +7320,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t xml:space="preserve">B3SA3 - B3          </t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
@@ -7321,13 +7329,13 @@
         </is>
       </c>
       <c r="F190" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="G190" t="n">
-        <v>0.028</v>
+        <v>1.156</v>
       </c>
       <c r="H190" t="n">
-        <v>1.4</v>
+        <v>18.49</v>
       </c>
     </row>
     <row r="191">
@@ -7338,17 +7346,17 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>07/10/2022</t>
+          <t>14/12/2022</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Juros Sobre Capital Próprio</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t xml:space="preserve">B3SA3 - B3          </t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -7357,13 +7365,13 @@
         </is>
       </c>
       <c r="F191" t="n">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="G191" t="n">
-        <v>0.055</v>
+        <v>0.1</v>
       </c>
       <c r="H191" t="n">
-        <v>2.32</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="192">
@@ -7374,7 +7382,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>20/09/2022</t>
+          <t>07/10/2022</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -7384,7 +7392,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t xml:space="preserve">B3SA3 - B3          </t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -7393,13 +7401,13 @@
         </is>
       </c>
       <c r="F192" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="G192" t="n">
-        <v>3.366</v>
+        <v>0.028</v>
       </c>
       <c r="H192" t="n">
-        <v>53.85</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="193">
@@ -7410,17 +7418,17 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>14/09/2022</t>
+          <t>07/10/2022</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Juros Sobre Capital Próprio</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t xml:space="preserve">B3SA3 - B3          </t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
@@ -7429,13 +7437,13 @@
         </is>
       </c>
       <c r="F193" t="n">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="G193" t="n">
-        <v>0.09</v>
+        <v>0.055</v>
       </c>
       <c r="H193" t="n">
-        <v>0.99</v>
+        <v>2.32</v>
       </c>
     </row>
     <row r="194">
@@ -7446,17 +7454,17 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>13/09/2022</t>
+          <t>20/09/2022</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Transferência - Liquidação</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>VALE3 - VALE S.A.</t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
@@ -7465,13 +7473,13 @@
         </is>
       </c>
       <c r="F194" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="G194" t="n">
-        <v>66.82299999999999</v>
+        <v>3.366</v>
       </c>
       <c r="H194" t="n">
-        <v>200.47</v>
+        <v>53.85</v>
       </c>
     </row>
     <row r="195">
@@ -7482,17 +7490,17 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>09/09/2022</t>
+          <t>14/09/2022</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Leilão de Fração</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>GOGL35 - ALPHABET INC.</t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
@@ -7501,13 +7509,13 @@
         </is>
       </c>
       <c r="F195" t="n">
-        <v>0.6</v>
+        <v>11</v>
       </c>
       <c r="G195" t="n">
-        <v>46.042</v>
+        <v>0.09</v>
       </c>
       <c r="H195" t="n">
-        <v>27.62</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="196">
@@ -7518,12 +7526,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>01/09/2022</t>
+          <t>13/09/2022</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Transferência - Liquidação</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -7537,13 +7545,13 @@
         </is>
       </c>
       <c r="F196" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G196" t="n">
-        <v>2.033</v>
+        <v>66.82299999999999</v>
       </c>
       <c r="H196" t="n">
-        <v>2.03</v>
+        <v>200.47</v>
       </c>
     </row>
     <row r="197">
@@ -7554,17 +7562,17 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>01/09/2022</t>
+          <t>09/09/2022</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Juros Sobre Capital Próprio</t>
+          <t>Leilão de Fração</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>VALE3 - VALE S.A.</t>
+          <t>GOGL35 - ALPHABET INC.</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
@@ -7573,34 +7581,34 @@
         </is>
       </c>
       <c r="F197" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="G197" t="n">
-        <v>1.539</v>
+        <v>46.042</v>
       </c>
       <c r="H197" t="n">
-        <v>1.3</v>
+        <v>27.62</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Debito</t>
+          <t>Credito</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>31/08/2022</t>
+          <t>01/09/2022</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Fração em Ativos</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>GOGL35 - ALPHABET INC.</t>
+          <t>VALE3 - VALE S.A.</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
@@ -7609,17 +7617,13 @@
         </is>
       </c>
       <c r="F198" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G198" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H198" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="G198" t="n">
+        <v>2.033</v>
+      </c>
+      <c r="H198" t="n">
+        <v>2.03</v>
       </c>
     </row>
     <row r="199">
@@ -7630,17 +7634,17 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>31/08/2022</t>
+          <t>01/09/2022</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Juros Sobre Capital Próprio</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t>VALE3 - VALE S.A.</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
@@ -7649,19 +7653,19 @@
         </is>
       </c>
       <c r="F199" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G199" t="n">
-        <v>2.939</v>
+        <v>1.539</v>
       </c>
       <c r="H199" t="n">
-        <v>47.02</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Credito</t>
+          <t>Debito</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -7671,12 +7675,12 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Juros Sobre Capital Próprio</t>
+          <t>Fração em Ativos</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t>GOGL35 - ALPHABET INC.</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -7685,13 +7689,17 @@
         </is>
       </c>
       <c r="F200" t="n">
-        <v>16</v>
-      </c>
-      <c r="G200" t="n">
-        <v>0.427</v>
-      </c>
-      <c r="H200" t="n">
-        <v>5.81</v>
+        <v>0.6</v>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="201">
@@ -7702,17 +7710,17 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>30/08/2022</t>
+          <t>31/08/2022</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Grupamento</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>GOGL35 - ALPHABET INC.</t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -7721,17 +7729,13 @@
         </is>
       </c>
       <c r="F201" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="G201" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H201" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>16</v>
+      </c>
+      <c r="G201" t="n">
+        <v>2.939</v>
+      </c>
+      <c r="H201" t="n">
+        <v>47.02</v>
       </c>
     </row>
     <row r="202">
@@ -7742,12 +7746,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>22/07/2022</t>
+          <t>31/08/2022</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Transferência - Liquidação</t>
+          <t>Juros Sobre Capital Próprio</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -7761,13 +7765,13 @@
         </is>
       </c>
       <c r="F202" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="G202" t="n">
-        <v>29.14</v>
+        <v>0.427</v>
       </c>
       <c r="H202" t="n">
-        <v>29.14</v>
+        <v>5.81</v>
       </c>
     </row>
     <row r="203">
@@ -7778,17 +7782,17 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>20/07/2022</t>
+          <t>30/08/2022</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Grupamento</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t>GOGL35 - ALPHABET INC.</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -7797,13 +7801,17 @@
         </is>
       </c>
       <c r="F203" t="n">
-        <v>15</v>
-      </c>
-      <c r="G203" t="n">
-        <v>1.858</v>
-      </c>
-      <c r="H203" t="n">
-        <v>27.86</v>
+        <v>17.6</v>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="204">
@@ -7814,17 +7822,17 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>19/07/2022</t>
+          <t>22/07/2022</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Desdobro</t>
+          <t>Transferência - Liquidação</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>GOGL35 - ALPHABET INC.</t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -7833,17 +7841,13 @@
         </is>
       </c>
       <c r="F204" t="n">
-        <v>209</v>
-      </c>
-      <c r="G204" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H204" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="G204" t="n">
+        <v>29.14</v>
+      </c>
+      <c r="H204" t="n">
+        <v>29.14</v>
       </c>
     </row>
     <row r="205">
@@ -7854,7 +7858,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>08/07/2022</t>
+          <t>20/07/2022</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -7864,7 +7868,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
@@ -7873,13 +7877,13 @@
         </is>
       </c>
       <c r="F205" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="G205" t="n">
-        <v>0.07000000000000001</v>
+        <v>1.858</v>
       </c>
       <c r="H205" t="n">
-        <v>3.49</v>
+        <v>27.86</v>
       </c>
     </row>
     <row r="206">
@@ -7890,17 +7894,17 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>08/07/2022</t>
+          <t>19/07/2022</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Juros Sobre Capital Próprio</t>
+          <t>Desdobro</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
+          <t>GOGL35 - ALPHABET INC.</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -7909,13 +7913,17 @@
         </is>
       </c>
       <c r="F206" t="n">
-        <v>50</v>
-      </c>
-      <c r="G206" t="n">
-        <v>0.061</v>
-      </c>
-      <c r="H206" t="n">
-        <v>2.58</v>
+        <v>209</v>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="207">
@@ -7926,17 +7934,17 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>20/06/2022</t>
+          <t>08/07/2022</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Juros Sobre Capital Próprio</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -7945,13 +7953,13 @@
         </is>
       </c>
       <c r="F207" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="G207" t="n">
-        <v>0.43</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H207" t="n">
-        <v>5.48</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="208">
@@ -7962,17 +7970,17 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>20/06/2022</t>
+          <t>08/07/2022</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Juros Sobre Capital Próprio</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
@@ -7981,13 +7989,13 @@
         </is>
       </c>
       <c r="F208" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="G208" t="n">
-        <v>1.428</v>
+        <v>0.061</v>
       </c>
       <c r="H208" t="n">
-        <v>21.41</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="209">
@@ -7998,17 +8006,17 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>15/06/2022</t>
+          <t>20/06/2022</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Juros Sobre Capital Próprio</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
@@ -8017,13 +8025,13 @@
         </is>
       </c>
       <c r="F209" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G209" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.43</v>
       </c>
       <c r="H209" t="n">
-        <v>0.95</v>
+        <v>5.48</v>
       </c>
     </row>
     <row r="210">
@@ -8034,12 +8042,12 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>16/05/2022</t>
+          <t>20/06/2022</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Rendimento</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -8056,10 +8064,10 @@
         <v>15</v>
       </c>
       <c r="G210" t="n">
-        <v>0.109</v>
+        <v>1.428</v>
       </c>
       <c r="H210" t="n">
-        <v>1.27</v>
+        <v>21.41</v>
       </c>
     </row>
     <row r="211">
@@ -8070,7 +8078,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>16/05/2022</t>
+          <t>15/06/2022</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -8080,7 +8088,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
@@ -8089,13 +8097,13 @@
         </is>
       </c>
       <c r="F211" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G211" t="n">
-        <v>2.861</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="H211" t="n">
-        <v>42.91</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="212">
@@ -8106,17 +8114,17 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>08/04/2022</t>
+          <t>16/05/2022</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Rendimento</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -8125,13 +8133,13 @@
         </is>
       </c>
       <c r="F212" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="G212" t="n">
-        <v>0.131</v>
+        <v>0.109</v>
       </c>
       <c r="H212" t="n">
-        <v>6.55</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="213">
@@ -8142,17 +8150,17 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>08/04/2022</t>
+          <t>16/05/2022</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Juros Sobre Capital Próprio</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
@@ -8161,13 +8169,13 @@
         </is>
       </c>
       <c r="F213" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="G213" t="n">
-        <v>0.05</v>
+        <v>2.861</v>
       </c>
       <c r="H213" t="n">
-        <v>2.13</v>
+        <v>42.91</v>
       </c>
     </row>
     <row r="214">
@@ -8178,17 +8186,17 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>25/03/2022</t>
+          <t>08/04/2022</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Transferência - Liquidação</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
+          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
@@ -8197,13 +8205,13 @@
         </is>
       </c>
       <c r="F214" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="G214" t="n">
-        <v>31.9</v>
+        <v>0.131</v>
       </c>
       <c r="H214" t="n">
-        <v>478.5</v>
+        <v>6.55</v>
       </c>
     </row>
     <row r="215">
@@ -8214,17 +8222,17 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>16/03/2022</t>
+          <t>08/04/2022</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Juros Sobre Capital Próprio</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
@@ -8233,13 +8241,13 @@
         </is>
       </c>
       <c r="F215" t="n">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="G215" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.05</v>
       </c>
       <c r="H215" t="n">
-        <v>0.96</v>
+        <v>2.13</v>
       </c>
     </row>
     <row r="216">
@@ -8250,17 +8258,17 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>16/03/2022</t>
+          <t>25/03/2022</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Transferência - Liquidação</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>VALE3 - VALE S.A.</t>
+          <t>PETR4 - PETROLEO BRASILEIRO S/A - PETROBRAS</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
@@ -8269,13 +8277,13 @@
         </is>
       </c>
       <c r="F216" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G216" t="n">
-        <v>3.719</v>
+        <v>31.9</v>
       </c>
       <c r="H216" t="n">
-        <v>3.71</v>
+        <v>478.5</v>
       </c>
     </row>
     <row r="217">
@@ -8286,17 +8294,17 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>09/02/2022</t>
+          <t>16/03/2022</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Transferência - Liquidação</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>VALE3 - VALE S.A.</t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
@@ -8305,13 +8313,13 @@
         </is>
       </c>
       <c r="F217" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="G217" t="n">
-        <v>90</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="H217" t="n">
-        <v>90</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="218">
@@ -8322,17 +8330,17 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>28/01/2022</t>
+          <t>16/03/2022</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Transferência - Liquidação</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>GOGL35 - ALPHABET INC.</t>
+          <t>VALE3 - VALE S.A.</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
@@ -8344,10 +8352,10 @@
         <v>1</v>
       </c>
       <c r="G218" t="n">
-        <v>94</v>
+        <v>3.719</v>
       </c>
       <c r="H218" t="n">
-        <v>94</v>
+        <v>3.71</v>
       </c>
     </row>
     <row r="219">
@@ -8358,7 +8366,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>28/01/2022</t>
+          <t>09/02/2022</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -8368,7 +8376,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>VALE3 - VALE S.A.</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
@@ -8380,10 +8388,10 @@
         <v>1</v>
       </c>
       <c r="G219" t="n">
-        <v>69.8</v>
+        <v>90</v>
       </c>
       <c r="H219" t="n">
-        <v>69.8</v>
+        <v>90</v>
       </c>
     </row>
     <row r="220">
@@ -8394,7 +8402,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>26/01/2022</t>
+          <t>28/01/2022</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -8404,7 +8412,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>GOGL35 - ALPHABET INC.</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
@@ -8413,13 +8421,13 @@
         </is>
       </c>
       <c r="F220" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G220" t="n">
-        <v>66</v>
+        <v>94</v>
       </c>
       <c r="H220" t="n">
-        <v>198</v>
+        <v>94</v>
       </c>
     </row>
     <row r="221">
@@ -8430,7 +8438,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>25/01/2022</t>
+          <t>28/01/2022</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -8440,7 +8448,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>GOGL35 - ALPHABET INC.</t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
@@ -8449,13 +8457,13 @@
         </is>
       </c>
       <c r="F221" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G221" t="n">
-        <v>96</v>
+        <v>69.8</v>
       </c>
       <c r="H221" t="n">
-        <v>288</v>
+        <v>69.8</v>
       </c>
     </row>
     <row r="222">
@@ -8466,7 +8474,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>24/01/2022</t>
+          <t>26/01/2022</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -8476,7 +8484,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>GOGL35 - ALPHABET INC.</t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
@@ -8485,13 +8493,13 @@
         </is>
       </c>
       <c r="F222" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G222" t="n">
-        <v>99.3</v>
+        <v>66</v>
       </c>
       <c r="H222" t="n">
-        <v>198.6</v>
+        <v>198</v>
       </c>
     </row>
     <row r="223">
@@ -8502,7 +8510,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>24/01/2022</t>
+          <t>25/01/2022</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -8512,7 +8520,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>GOGL35 - ALPHABET INC.</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -8521,13 +8529,13 @@
         </is>
       </c>
       <c r="F223" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G223" t="n">
-        <v>69.92</v>
+        <v>96</v>
       </c>
       <c r="H223" t="n">
-        <v>69.92</v>
+        <v>288</v>
       </c>
     </row>
     <row r="224">
@@ -8538,7 +8546,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>21/01/2022</t>
+          <t>24/01/2022</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -8548,7 +8556,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>GOGL35 - ALPHABET INC.</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
@@ -8557,13 +8565,13 @@
         </is>
       </c>
       <c r="F224" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G224" t="n">
-        <v>69.87</v>
+        <v>99.3</v>
       </c>
       <c r="H224" t="n">
-        <v>69.87</v>
+        <v>198.6</v>
       </c>
     </row>
     <row r="225">
@@ -8574,17 +8582,17 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>07/01/2022</t>
+          <t>24/01/2022</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Juros Sobre Capital Próprio</t>
+          <t>Transferência - Liquidação</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
@@ -8593,13 +8601,13 @@
         </is>
       </c>
       <c r="F225" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G225" t="n">
-        <v>0.05</v>
+        <v>69.92</v>
       </c>
       <c r="H225" t="n">
-        <v>1.05</v>
+        <v>69.92</v>
       </c>
     </row>
     <row r="226">
@@ -8610,7 +8618,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>07/01/2022</t>
+          <t>21/01/2022</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -8620,7 +8628,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>GOGL35 - ALPHABET INC.</t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
@@ -8629,13 +8637,13 @@
         </is>
       </c>
       <c r="F226" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G226" t="n">
-        <v>107.03</v>
+        <v>69.87</v>
       </c>
       <c r="H226" t="n">
-        <v>214.06</v>
+        <v>69.87</v>
       </c>
     </row>
     <row r="227">
@@ -8651,12 +8659,12 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Transferência - Liquidação</t>
+          <t>Juros Sobre Capital Próprio</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
@@ -8665,13 +8673,13 @@
         </is>
       </c>
       <c r="F227" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="G227" t="n">
-        <v>75.95999999999999</v>
+        <v>0.05</v>
       </c>
       <c r="H227" t="n">
-        <v>227.88</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="228">
@@ -8682,7 +8690,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>05/01/2022</t>
+          <t>07/01/2022</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -8692,7 +8700,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
+          <t>GOGL35 - ALPHABET INC.</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
@@ -8701,13 +8709,13 @@
         </is>
       </c>
       <c r="F228" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="G228" t="n">
-        <v>10.79</v>
+        <v>107.03</v>
       </c>
       <c r="H228" t="n">
-        <v>269.75</v>
+        <v>214.06</v>
       </c>
     </row>
     <row r="229">
@@ -8718,7 +8726,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>30/12/2021</t>
+          <t>07/01/2022</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -8728,7 +8736,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
@@ -8737,13 +8745,13 @@
         </is>
       </c>
       <c r="F229" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="G229" t="n">
-        <v>11.17</v>
+        <v>75.95999999999999</v>
       </c>
       <c r="H229" t="n">
-        <v>189.92</v>
+        <v>227.88</v>
       </c>
     </row>
     <row r="230">
@@ -8754,7 +8762,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>29/12/2021</t>
+          <t>05/01/2022</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -8773,13 +8781,13 @@
         </is>
       </c>
       <c r="F230" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="G230" t="n">
-        <v>11.32</v>
+        <v>10.79</v>
       </c>
       <c r="H230" t="n">
-        <v>90.56999999999999</v>
+        <v>269.75</v>
       </c>
     </row>
     <row r="231">
@@ -8790,17 +8798,17 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>15/12/2021</t>
+          <t>30/12/2021</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Dividendo</t>
+          <t>Transferência - Liquidação</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
@@ -8809,13 +8817,13 @@
         </is>
       </c>
       <c r="F231" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="G231" t="n">
-        <v>0.09</v>
+        <v>11.17</v>
       </c>
       <c r="H231" t="n">
-        <v>0.09</v>
+        <v>189.92</v>
       </c>
     </row>
     <row r="232">
@@ -8826,7 +8834,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>30/11/2021</t>
+          <t>29/12/2021</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -8836,7 +8844,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>GOGL35 - ALPHABET INC.</t>
+          <t>B3SA3 - B3 S.A. - BRASIL, BOLSA, BALCÃO</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
@@ -8845,13 +8853,13 @@
         </is>
       </c>
       <c r="F232" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G232" t="n">
-        <v>107.25</v>
+        <v>11.32</v>
       </c>
       <c r="H232" t="n">
-        <v>107.25</v>
+        <v>90.56999999999999</v>
       </c>
     </row>
     <row r="233">
@@ -8862,17 +8870,17 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>26/11/2021</t>
+          <t>15/12/2021</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Transferência - Liquidação</t>
+          <t>Dividendo</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>GOGL35 - ALPHABET INC.</t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -8884,10 +8892,10 @@
         <v>1</v>
       </c>
       <c r="G233" t="n">
-        <v>109.07</v>
+        <v>0.09</v>
       </c>
       <c r="H233" t="n">
-        <v>109.07</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="234">
@@ -8898,7 +8906,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>22/11/2021</t>
+          <t>30/11/2021</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -8908,7 +8916,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>GOGL35 - ALPHABET INC.</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
@@ -8920,10 +8928,10 @@
         <v>1</v>
       </c>
       <c r="G234" t="n">
-        <v>79.15000000000001</v>
+        <v>107.25</v>
       </c>
       <c r="H234" t="n">
-        <v>79.15000000000001</v>
+        <v>107.25</v>
       </c>
     </row>
     <row r="235">
@@ -8934,7 +8942,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>18/11/2021</t>
+          <t>26/11/2021</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -8944,7 +8952,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>MSFT34 - MICROSOFT CORPORATION</t>
+          <t>GOGL35 - ALPHABET INC.</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
@@ -8956,10 +8964,10 @@
         <v>1</v>
       </c>
       <c r="G235" t="n">
-        <v>76.28</v>
+        <v>109.07</v>
       </c>
       <c r="H235" t="n">
-        <v>76.28</v>
+        <v>109.07</v>
       </c>
     </row>
     <row r="236">
@@ -8970,7 +8978,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>10/11/2021</t>
+          <t>22/11/2021</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -8980,7 +8988,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>GOGL35 - ALPHABET INC.</t>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -8992,9 +9000,81 @@
         <v>1</v>
       </c>
       <c r="G236" t="n">
+        <v>79.15000000000001</v>
+      </c>
+      <c r="H236" t="n">
+        <v>79.15000000000001</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Credito</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>18/11/2021</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Transferência - Liquidação</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>MSFT34 - MICROSOFT CORPORATION</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>NU INVEST CORRETORA DE VALORES S.A.</t>
+        </is>
+      </c>
+      <c r="F237" t="n">
+        <v>1</v>
+      </c>
+      <c r="G237" t="n">
+        <v>76.28</v>
+      </c>
+      <c r="H237" t="n">
+        <v>76.28</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Credito</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>10/11/2021</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Transferência - Liquidação</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>GOGL35 - ALPHABET INC.</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>NU INVEST CORRETORA DE VALORES S.A.</t>
+        </is>
+      </c>
+      <c r="F238" t="n">
+        <v>1</v>
+      </c>
+      <c r="G238" t="n">
         <v>111.52</v>
       </c>
-      <c r="H236" t="n">
+      <c r="H238" t="n">
         <v>111.52</v>
       </c>
     </row>

</xml_diff>